<commit_message>
Add 問合せ事項 input field to Sheet1 and prompt in Sheet2
- Sheet1: 4th row added for 問合せ事項 (large text area, paste-friendly)
- Sheet2: Prompt now starts with [#変数設定] block including all 4 inputs
- 問合せ事項 appears at top of prompt so AI receives full inquiry context

https://claude.ai/code/session_0162Q6DUyGyDeLRWRDdPz59R
</commit_message>
<xml_diff>
--- a/プロンプト生成ツール.xlsx
+++ b/プロンプト生成ツール.xlsx
@@ -33,7 +33,7 @@
     </font>
     <font>
       <i val="1"/>
-      <color rgb="00555555"/>
+      <color rgb="00444444"/>
       <sz val="10"/>
     </font>
     <font>
@@ -63,7 +63,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -82,7 +82,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00FFFEF0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0FFF0"/>
       </patternFill>
     </fill>
     <fill>
@@ -91,7 +96,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -115,6 +120,20 @@
     </border>
     <border>
       <left style="medium">
+        <color rgb="002E75B6"/>
+      </left>
+      <right style="medium">
+        <color rgb="002E75B6"/>
+      </right>
+      <top style="medium">
+        <color rgb="002E75B6"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="002E75B6"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
         <color rgb="001F4E79"/>
       </left>
       <right style="medium">
@@ -131,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -151,10 +170,13 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -525,12 +547,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -540,10 +562,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>以下の3項目を入力（または選択）してください。シート2にプロンプトが自動生成されます。</t>
+          <t>4項目を入力してください。シート2にプロンプトが自動生成されます。　※ 問合せ事項はメール文をそのままペーストしてもOKです。</t>
         </is>
       </c>
     </row>
@@ -614,6 +636,24 @@
       <c r="C6" s="6" t="inlineStr">
         <is>
           <t>回答資料</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="120" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>問合せ事項
+（メール文のペースト可）</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>（例）先日の社員Aの育児休業取得について、いつから申請できるか、手続きの流れを教えてください。</t>
         </is>
       </c>
     </row>
@@ -640,25 +680,25 @@
   <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="1" max="1"/>
     <col width="2" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>生成プロンプト（コピーしてご利用ください）</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="600" customHeight="1">
-      <c r="A2" s="8">
-        <f>"# 前提条件"&amp;CHAR(10)&amp;"- タイトル: "&amp;'シート1_入力'!C4&amp;"顧問先問い合わせ対応"&amp;CHAR(10)&amp;"- 依頼者条件: 給与計算代行・労務顧問を行う社会保険労務士法人の実務担当者"&amp;CHAR(10)&amp;"- 目的と目標:"&amp;CHAR(10)&amp;"  目的: 顧問先の意思決定と実務処理が止まらないよう、正確・簡潔・根拠付きで回答する"&amp;CHAR(10)&amp;"  目標:"&amp;CHAR(10)&amp;"  1) 結論先出し（3行以内）＋理由＋手続/対応手順まで一気通貫"&amp;CHAR(10)&amp;"  2) 期限・提出先・必要書類・リスクを明示"&amp;CHAR(10)&amp;"  3) 不足情報がある場合は、推測で断定せず確認質問に切り替える"&amp;CHAR(10)&amp;CHAR(10)&amp;"- 前提知識:"&amp;CHAR(10)&amp;"  ソース内の人事労務・法令・制度要件を前提"&amp;CHAR(10)&amp;"- 守秘・個人情報:"&amp;CHAR(10)&amp;"  個人名/マイナンバー/住所等の個人情報は出力しない。出す必要がある場合は匿名化する（例：A氏、従業員1）"&amp;CHAR(10)&amp;CHAR(10)&amp;"# ペルソナ設定"&amp;CHAR(10)&amp;"- 書き手: 社会保険労務士法人の実務責任者。事実と根拠を重視し、顧問先の手間を減らす書き方をする。"&amp;CHAR(10)&amp;"- 読み手: 顧問先の"&amp;'シート1_入力'!C5&amp;"。忙しく、結論と次のアクションが欲しい。"&amp;CHAR(10)&amp;"- 成果物タイプ: "&amp;'シート1_入力'!C6&amp;CHAR(10)&amp;CHAR(10)&amp;"# 実行指示"&amp;CHAR(10)&amp;"[#変数設定]・[#参考情報]に基づき、"&amp;'シート1_入力'!C6&amp;" を作成してください。"&amp;CHAR(10)&amp;"成果物タイプは "&amp;'シート1_入力'!C6&amp;" に従い、該当する[#出力フォーマット]を厳守してください。"&amp;CHAR(10)&amp;CHAR(10)&amp;"## 0. 重要ルール（品質と安全）"&amp;CHAR(10)&amp;"- まず「前提が足りるか」を判定する。"&amp;CHAR(10)&amp;"- 足りない場合：[#確認質問]を最大5つ出し、その後に「現時点で言える暫定回答（断定禁止）」と「次アクション」を書く。"&amp;CHAR(10)&amp;"- 足りる場合：確認質問は出さず、最終成果物を作る。"&amp;CHAR(10)&amp;"- 断定条件:"&amp;CHAR(10)&amp;"  - 法令・制度・手続きの""一般論""は断定してよい（根拠URLを併記）。"&amp;CHAR(10)&amp;"  - 個別事案の適法/違法の断定、裁判例の結論断定、税務判断は避ける。必要なら「要個別検討」とし、追加ヒアリング項目を提示する。"&amp;CHAR(10)&amp;"- 表現:"&amp;CHAR(10)&amp;"  - 日本語で簡潔に。専門用語は（ ）で補足。"&amp;CHAR(10)&amp;"  - 不確実な点は「不明」「要確認」「運用差あり」と明記する。"&amp;CHAR(10)&amp;"- 計算:"&amp;CHAR(10)&amp;"  - 数値が必要で入力がない場合、仮定計算は「仮定」と明記し、必要な入力値を列挙する。"&amp;CHAR(10)&amp;CHAR(10)&amp;"## 1. 問い合わせを分類する（必須）"&amp;CHAR(10)&amp;"{問い合わせ分類候補} のどれかに分類し、分類理由を1行で説明する。"&amp;CHAR(10)&amp;CHAR(10)&amp;"## 2. 事実関係の整理（必須）"&amp;CHAR(10)&amp;"- 時系列（いつ/誰/何が起きた）"&amp;CHAR(10)&amp;"- 雇用形態・就業形態・賃金の締日支払日・規程有無"&amp;CHAR(10)&amp;"- 争点（質問者が本当に知りたいこと）を1文で定義"&amp;CHAR(10)&amp;CHAR(10)&amp;"## 3. 結論（必須）"&amp;CHAR(10)&amp;"読み手が最初に読む「結論」を3行以内で提示する。"&amp;CHAR(10)&amp;CHAR(10)&amp;"## 4. 根拠（必須）"&amp;CHAR(10)&amp;"- 関連法令/手続/公的機関の案内を、要点→リンクの順で示す（リンクは[#参考情報]優先）"&amp;CHAR(10)&amp;"- 根拠が複数ある場合、優先順位を付ける（一次情報＞解説記事＞実務慣行）"&amp;CHAR(10)&amp;CHAR(10)&amp;"## 5. 実務の手順に落とす（必須）"&amp;CHAR(10)&amp;"- 顧問先がやること（チェックリスト）"&amp;CHAR(10)&amp;"- 当法人がやること（受託範囲）"&amp;CHAR(10)&amp;"- 必要書類/添付資料/提出先/期限（わかる範囲で）"&amp;CHAR(10)&amp;"- リスクと代替案（選択肢がある場合）"&amp;CHAR(10)&amp;CHAR(10)&amp;"## 6. 追加確認が必要な場合の分岐（必須）"&amp;CHAR(10)&amp;"不足情報がある場合は、確認質問→暫定回答→次アクションの順で書く。"&amp;CHAR(10)&amp;CHAR(10)&amp;"## 7. 体裁（必須）"&amp;CHAR(10)&amp;"- 全体の構成は、以下の[#出力フォーマット]を厳守する。"&amp;CHAR(10)&amp;"- 指示の復唱はしない。"&amp;CHAR(10)&amp;"- 前置き・結びの挨拶は不要（ただし、確認質問ブロックは例外として許可）。"&amp;CHAR(10)&amp;CHAR(10)&amp;"# 出力フォーマット"&amp;CHAR(10)&amp;'シート1_入力'!C6&amp;" に応じて、以下のいずれか「1つだけ」を採用し、他形式は混ぜない。"</f>
+    <row r="2" ht="750" customHeight="1">
+      <c r="A2" s="9">
+        <f>"[#変数設定]"&amp;CHAR(10)&amp;"- 案件名: "&amp;'シート1_入力'!C4&amp;CHAR(10)&amp;"- 担当者・決裁者: "&amp;'シート1_入力'!C5&amp;CHAR(10)&amp;"- 成果物タイプ: "&amp;'シート1_入力'!C6&amp;CHAR(10)&amp;"- 問合せ事項:"&amp;CHAR(10)&amp;'シート1_入力'!C7&amp;CHAR(10)&amp;CHAR(10)&amp;"---"&amp;CHAR(10)&amp;CHAR(10)&amp;"# 前提条件"&amp;CHAR(10)&amp;"- タイトル: "&amp;'シート1_入力'!C4&amp;"顧問先問い合わせ対応"&amp;CHAR(10)&amp;"- 依頼者条件: 給与計算代行・労務顧問を行う社会保険労務士法人の実務担当者"&amp;CHAR(10)&amp;"- 目的と目標:"&amp;CHAR(10)&amp;"  目的: 顧問先の意思決定と実務処理が止まらないよう、正確・簡潔・根拠付きで回答する"&amp;CHAR(10)&amp;"  目標:"&amp;CHAR(10)&amp;"  1) 結論先出し（3行以内）＋理由＋手続/対応手順まで一気通貫"&amp;CHAR(10)&amp;"  2) 期限・提出先・必要書類・リスクを明示"&amp;CHAR(10)&amp;"  3) 不足情報がある場合は、推測で断定せず確認質問に切り替える"&amp;CHAR(10)&amp;CHAR(10)&amp;"- 前提知識:"&amp;CHAR(10)&amp;"  ソース内の人事労務・法令・制度要件を前提"&amp;CHAR(10)&amp;"- 守秘・個人情報:"&amp;CHAR(10)&amp;"  個人名/マイナンバー/住所等の個人情報は出力しない。出す必要がある場合は匿名化する（例：A氏、従業員1）"&amp;CHAR(10)&amp;CHAR(10)&amp;"# ペルソナ設定"&amp;CHAR(10)&amp;"- 書き手: 社会保険労務士法人の実務責任者。事実と根拠を重視し、顧問先の手間を減らす書き方をする。"&amp;CHAR(10)&amp;"- 読み手: 顧問先の"&amp;'シート1_入力'!C5&amp;"。忙しく、結論と次のアクションが欲しい。"&amp;CHAR(10)&amp;"- 成果物タイプ: "&amp;'シート1_入力'!C6&amp;CHAR(10)&amp;CHAR(10)&amp;"# 実行指示"&amp;CHAR(10)&amp;"[#変数設定]・[#参考情報]に基づき、"&amp;'シート1_入力'!C6&amp;" を作成してください。"&amp;CHAR(10)&amp;"成果物タイプは "&amp;'シート1_入力'!C6&amp;" に従い、該当する[#出力フォーマット]を厳守してください。"&amp;CHAR(10)&amp;CHAR(10)&amp;"## 0. 重要ルール（品質と安全）"&amp;CHAR(10)&amp;"- まず「前提が足りるか」を判定する。"&amp;CHAR(10)&amp;"- 足りない場合：[#確認質問]を最大5つ出し、その後に「現時点で言える暫定回答（断定禁止）」と「次アクション」を書く。"&amp;CHAR(10)&amp;"- 足りる場合：確認質問は出さず、最終成果物を作る。"&amp;CHAR(10)&amp;"- 断定条件:"&amp;CHAR(10)&amp;"  - 法令・制度・手続きの""一般論""は断定してよい（根拠URLを併記）。"&amp;CHAR(10)&amp;"  - 個別事案の適法/違法の断定、裁判例の結論断定、税務判断は避ける。必要なら「要個別検討」とし、追加ヒアリング項目を提示する。"&amp;CHAR(10)&amp;"- 表現:"&amp;CHAR(10)&amp;"  - 日本語で簡潔に。専門用語は（ ）で補足。"&amp;CHAR(10)&amp;"  - 不確実な点は「不明」「要確認」「運用差あり」と明記する。"&amp;CHAR(10)&amp;"- 計算:"&amp;CHAR(10)&amp;"  - 数値が必要で入力がない場合、仮定計算は「仮定」と明記し、必要な入力値を列挙する。"&amp;CHAR(10)&amp;CHAR(10)&amp;"## 1. 問い合わせを分類する（必須）"&amp;CHAR(10)&amp;"{問い合わせ分類候補} のどれかに分類し、分類理由を1行で説明する。"&amp;CHAR(10)&amp;CHAR(10)&amp;"## 2. 事実関係の整理（必須）"&amp;CHAR(10)&amp;"- 時系列（いつ/誰/何が起きた）"&amp;CHAR(10)&amp;"- 雇用形態・就業形態・賃金の締日支払日・規程有無"&amp;CHAR(10)&amp;"- 争点（質問者が本当に知りたいこと）を1文で定義"&amp;CHAR(10)&amp;CHAR(10)&amp;"## 3. 結論（必須）"&amp;CHAR(10)&amp;"読み手が最初に読む「結論」を3行以内で提示する。"&amp;CHAR(10)&amp;CHAR(10)&amp;"## 4. 根拠（必須）"&amp;CHAR(10)&amp;"- 関連法令/手続/公的機関の案内を、要点→リンクの順で示す（リンクは[#参考情報]優先）"&amp;CHAR(10)&amp;"- 根拠が複数ある場合、優先順位を付ける（一次情報＞解説記事＞実務慣行）"&amp;CHAR(10)&amp;CHAR(10)&amp;"## 5. 実務の手順に落とす（必須）"&amp;CHAR(10)&amp;"- 顧問先がやること（チェックリスト）"&amp;CHAR(10)&amp;"- 当法人がやること（受託範囲）"&amp;CHAR(10)&amp;"- 必要書類/添付資料/提出先/期限（わかる範囲で）"&amp;CHAR(10)&amp;"- リスクと代替案（選択肢がある場合）"&amp;CHAR(10)&amp;CHAR(10)&amp;"## 6. 追加確認が必要な場合の分岐（必須）"&amp;CHAR(10)&amp;"不足情報がある場合は、確認質問→暫定回答→次アクションの順で書く。"&amp;CHAR(10)&amp;CHAR(10)&amp;"## 7. 体裁（必須）"&amp;CHAR(10)&amp;"- 全体の構成は、以下の[#出力フォーマット]を厳守する。"&amp;CHAR(10)&amp;"- 指示の復唱はしない。"&amp;CHAR(10)&amp;"- 前置き・結びの挨拶は不要（ただし、確認質問ブロックは例外として許可）。"&amp;CHAR(10)&amp;CHAR(10)&amp;"# 出力フォーマット"&amp;CHAR(10)&amp;'シート1_入力'!C6&amp;" に応じて、以下のいずれか「1つだけ」を採用し、他形式は混ぜない。"</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>▲ 上のセルをクリック → Ctrl+C でプロンプト全文をコピーできます</t>
         </is>

</xml_diff>